<commit_message>
ELA Word Chapter 2
</commit_message>
<xml_diff>
--- a/data/2026_F_M_Words.xlsx
+++ b/data/2026_F_M_Words.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\채아_SALT\2026_F\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\word-tester\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F0E715C-1533-4CC3-AA6C-230A8F3CE6A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C678FE01-E60E-4E03-B0AB-6BECF9843977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A78F504C-B3D1-44D7-A0F0-C4A481C15F08}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A78F504C-B3D1-44D7-A0F0-C4A481C15F08}"/>
   </bookViews>
   <sheets>
     <sheet name="Chapter 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Chapter 2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="218">
   <si>
     <t>단어 (Word)</t>
   </si>
@@ -417,6 +418,288 @@
   <si>
     <t>ask out</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>뜻 (Definition)</t>
+  </si>
+  <si>
+    <t>arrogant [adj.]</t>
+  </si>
+  <si>
+    <t>Showing too much pride in oneself</t>
+  </si>
+  <si>
+    <t>A feeling of too much pride in oneself</t>
+  </si>
+  <si>
+    <t>• Declaring that you are sure to win is another example of your arrogance.</t>
+  </si>
+  <si>
+    <t>boycott [v.]</t>
+  </si>
+  <si>
+    <t>To join others in refusing to support an organization</t>
+  </si>
+  <si>
+    <t>• Customers plan to boycott that store if it continues to discriminate.</t>
+  </si>
+  <si>
+    <t>campaign [v.]</t>
+  </si>
+  <si>
+    <t>To take part in actions planned to accomplish a particular goal</t>
+  </si>
+  <si>
+    <t>• Students who wish to campaign for class office must submit petitions.</t>
+  </si>
+  <si>
+    <t>ceremony [n.]</t>
+  </si>
+  <si>
+    <t>A formal event held in honor of a special occasion.</t>
+  </si>
+  <si>
+    <t>1) Control over and responsibility for care of something or someone</t>
+  </si>
+  <si>
+    <t>2) In the keeping of the police; in jail</t>
+  </si>
+  <si>
+    <t>degrade [v.]</t>
+  </si>
+  <si>
+    <t>To bring shame or disgrace upon</t>
+  </si>
+  <si>
+    <t>Causing shame or disgrace</t>
+  </si>
+  <si>
+    <t>detain [v.]</t>
+  </si>
+  <si>
+    <t>To stop or hold; to keep from going on</t>
+  </si>
+  <si>
+    <t>1) To reach out</t>
+  </si>
+  <si>
+    <t>• The conductor extended her arms as a signal to the orchestra to be ready.</t>
+  </si>
+  <si>
+    <t>2) To offer</t>
+  </si>
+  <si>
+    <t>• I wish to extend my apologies for behaving so badly.</t>
+  </si>
+  <si>
+    <t>3) To make longer</t>
+  </si>
+  <si>
+    <t>• The exhibition was so popular that the museum decided to extend it by a week.</t>
+  </si>
+  <si>
+    <t>4) To stretch or spread outward from a certain point</t>
+  </si>
+  <si>
+    <t>• The property extends for a half mile beyond the river.</t>
+  </si>
+  <si>
+    <t>integrate [v.]</t>
+  </si>
+  <si>
+    <t>To unite into a whole; especially to end the separation of people of different races</t>
+  </si>
+  <si>
+    <t>1) A noteworthy success</t>
+  </si>
+  <si>
+    <t>• The scientist's triumph was discovering a new medicine that helps people.</t>
+  </si>
+  <si>
+    <t>2) The joy that winning brings</t>
+  </si>
+  <si>
+    <t>• The dancer who was invited to audition shot a look of triumph at those who were not so lucky.</t>
+  </si>
+  <si>
+    <t>To win</t>
+  </si>
+  <si>
+    <t>• The winner of the national spelling bee triumphed over 49 other contestants.</t>
+  </si>
+  <si>
+    <t>Joyful over a victory or success</t>
+  </si>
+  <si>
+    <t>• The team felt triumphant after winning the championship game.</t>
+  </si>
+  <si>
+    <t>vacate [v.]</t>
+  </si>
+  <si>
+    <t>To make empty, as by leaving</t>
+  </si>
+  <si>
+    <t>1) The decision reached at the end of a trial</t>
+  </si>
+  <si>
+    <t>2) A judgment or opinion</t>
+  </si>
+  <si>
+    <t>1) To break, as a law or a promise</t>
+  </si>
+  <si>
+    <t>2) To treat in an improper or disrespectful way</t>
+  </si>
+  <si>
+    <t>• The vandals who violated the cemetery by knocking over gravestones had to restore it.</t>
+  </si>
+  <si>
+    <t>A breaking of or failing to keep something like a law or a promise.</t>
+  </si>
+  <si>
+    <t>• Throwing litter on the ground is a violation of the park’s rules.</t>
+  </si>
+  <si>
+    <t>1) To end a relationship or partnership.</t>
+  </si>
+  <si>
+    <t>• After a long conversation, Harry and Cho decided to break up and go their separate ways.</t>
+  </si>
+  <si>
+    <t>2) To separate or disperse something into smaller parts or pieces.</t>
+  </si>
+  <si>
+    <t>• The teacher asked the students to break up into smaller groups for the group project.</t>
+  </si>
+  <si>
+    <t>3) To interrupt or stop something, such as a gathering or activity.</t>
+  </si>
+  <si>
+    <t>• The principal came in to break up the argument between two students in the hallway.</t>
+  </si>
+  <si>
+    <t>1) To return something to its original place or owner.</t>
+  </si>
+  <si>
+    <t>• After borrowing the book from the library, Tim promised to bring it back by the due date.</t>
+  </si>
+  <si>
+    <t>2) To cause something to return or reappear, often something that was once popular or in use.</t>
+  </si>
+  <si>
+    <t>• The fashion store decided to bring back the popular style of jeans from the 90s.</t>
+  </si>
+  <si>
+    <t>3) To evoke memories or feelings about the past.</t>
+  </si>
+  <si>
+    <t>• The old photograph helped bring back memories of the family vacation from last summer.</t>
+  </si>
+  <si>
+    <t>• You were arrogant to claim that you knew all the answers. • The athlete was talented, but his arrogant attitude made it hard for others to like him.</t>
+  </si>
+  <si>
+    <t>• The bride and groom exchanged rings during the wedding ceremony. • The graduation ceremony will take place in the school gym next week. • There will be a ceremony to honor the firefighters for their bravery.</t>
+  </si>
+  <si>
+    <t>custody [n.] (Sense 1)</t>
+  </si>
+  <si>
+    <t>• The stolen Picasso painting was returned to the custody of the Museum of Modern Art. • After their parents separated, the court decided who would have custody of the children.</t>
+  </si>
+  <si>
+    <t>custody [n.] (Sense 2)</t>
+  </si>
+  <si>
+    <t>• The police officer took the thief into custody. • After the accident, the authorities took custody of the evidence for investigation.</t>
+  </si>
+  <si>
+    <t>• By lying to cover up his cheating, Sam degraded himself even more. • The teacher reminded us not to degrade our classmates by calling them names.</t>
+  </si>
+  <si>
+    <t>• Losing the trophy because one player cheated on a test was a degrading experience. • The graffiti on the school walls was degrading to the community.</t>
+  </si>
+  <si>
+    <t>• The hall monitor detained us until we could prove we had permission to leave the classroom. • The police had to detain the suspect to ask him more questions. • The meeting was supposed to end at 3 p.m., but several questions detained us.</t>
+  </si>
+  <si>
+    <t>extend [v.] (Sense 1)</t>
+  </si>
+  <si>
+    <t>extend [v.] (Sense 2)</t>
+  </si>
+  <si>
+    <t>extend [v.] (Sense 3)</t>
+  </si>
+  <si>
+    <t>extend [v.] (Sense 4)</t>
+  </si>
+  <si>
+    <t>• The town worked hard to integrate people from different cultures and backgrounds. • We need to integrate all of our ideas to create one final project.</t>
+  </si>
+  <si>
+    <t>triumph [n.] (Sense 1)</t>
+  </si>
+  <si>
+    <t>triumph [n.] (Sense 2)</t>
+  </si>
+  <si>
+    <t>• We will vacate the house at the end of June to make way for the people moving in. • The hotel asked guests to vacate their rooms by 11 a.m. on the day of departure. • During the evacuation drill, everyone practiced how to vacate the building quickly and safely. • The teacher asked the students to vacate their desks during the classroom renovation.</t>
+  </si>
+  <si>
+    <t>verdict [n.] (Sense 1)</t>
+  </si>
+  <si>
+    <t>• The jury looked grim as she announced the verdict. • The jury gave a verdict of "guilty" after hearing all the evidence in the trial.</t>
+  </si>
+  <si>
+    <t>verdict [n.] (Sense 2)</t>
+  </si>
+  <si>
+    <t>• The verdict on the new computer is that it does twice the work in half the time. • After the game, the coach gave his verdict on how the team performed.</t>
+  </si>
+  <si>
+    <t>violate [v.] (Sense 1)</t>
+  </si>
+  <si>
+    <t>• Damien violated our teacher’s trust by trying to cheat on the homework. • If you talk during a test, you might violate the rules of the classroom.</t>
+  </si>
+  <si>
+    <t>violate [v.] (Sense 2)</t>
+  </si>
+  <si>
+    <t>break up (Sense 1)</t>
+  </si>
+  <si>
+    <t>break up (Sense 2)</t>
+  </si>
+  <si>
+    <t>break up (Sense 3)</t>
+  </si>
+  <si>
+    <t>bring back (Sense 1)</t>
+  </si>
+  <si>
+    <t>bring back (Sense 2)</t>
+  </si>
+  <si>
+    <t>bring back (Sense 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">arrogance [n.]  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">degrading [adj.]  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">triumph [v.]  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">triumphant [adj.]  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">violation [n.]  </t>
   </si>
 </sst>
 </file>
@@ -1317,4 +1600,371 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A63C5D87-E957-48D6-B966-525BF50244A4}">
+  <dimension ref="A1:C32"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.875" customWidth="1"/>
+    <col min="2" max="2" width="29.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B6" t="s">
+        <v>136</v>
+      </c>
+      <c r="C6" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>185</v>
+      </c>
+      <c r="B7" t="s">
+        <v>137</v>
+      </c>
+      <c r="C7" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>187</v>
+      </c>
+      <c r="B8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C8" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B9" t="s">
+        <v>140</v>
+      </c>
+      <c r="C9" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>214</v>
+      </c>
+      <c r="B10" t="s">
+        <v>141</v>
+      </c>
+      <c r="C10" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>142</v>
+      </c>
+      <c r="B11" t="s">
+        <v>143</v>
+      </c>
+      <c r="C11" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>192</v>
+      </c>
+      <c r="B12" t="s">
+        <v>144</v>
+      </c>
+      <c r="C12" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>193</v>
+      </c>
+      <c r="B13" t="s">
+        <v>146</v>
+      </c>
+      <c r="C13" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>194</v>
+      </c>
+      <c r="B14" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>195</v>
+      </c>
+      <c r="B15" t="s">
+        <v>150</v>
+      </c>
+      <c r="C15" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>152</v>
+      </c>
+      <c r="B16" t="s">
+        <v>153</v>
+      </c>
+      <c r="C16" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>197</v>
+      </c>
+      <c r="B17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C17" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>198</v>
+      </c>
+      <c r="B18" t="s">
+        <v>156</v>
+      </c>
+      <c r="C18" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>215</v>
+      </c>
+      <c r="B19" t="s">
+        <v>158</v>
+      </c>
+      <c r="C19" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>216</v>
+      </c>
+      <c r="B20" t="s">
+        <v>160</v>
+      </c>
+      <c r="C20" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>162</v>
+      </c>
+      <c r="B21" t="s">
+        <v>163</v>
+      </c>
+      <c r="C21" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>200</v>
+      </c>
+      <c r="B22" t="s">
+        <v>164</v>
+      </c>
+      <c r="C22" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>202</v>
+      </c>
+      <c r="B23" t="s">
+        <v>165</v>
+      </c>
+      <c r="C23" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>204</v>
+      </c>
+      <c r="B24" t="s">
+        <v>166</v>
+      </c>
+      <c r="C24" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>206</v>
+      </c>
+      <c r="B25" t="s">
+        <v>167</v>
+      </c>
+      <c r="C25" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>217</v>
+      </c>
+      <c r="B26" t="s">
+        <v>169</v>
+      </c>
+      <c r="C26" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>207</v>
+      </c>
+      <c r="B27" t="s">
+        <v>171</v>
+      </c>
+      <c r="C27" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>208</v>
+      </c>
+      <c r="B28" t="s">
+        <v>173</v>
+      </c>
+      <c r="C28" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>209</v>
+      </c>
+      <c r="B29" t="s">
+        <v>175</v>
+      </c>
+      <c r="C29" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>210</v>
+      </c>
+      <c r="B30" t="s">
+        <v>177</v>
+      </c>
+      <c r="C30" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>211</v>
+      </c>
+      <c r="B31" t="s">
+        <v>179</v>
+      </c>
+      <c r="C31" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>212</v>
+      </c>
+      <c r="B32" t="s">
+        <v>181</v>
+      </c>
+      <c r="C32" t="s">
+        <v>182</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Remove part of speech from an excel file
</commit_message>
<xml_diff>
--- a/data/2026_F_M_Words.xlsx
+++ b/data/2026_F_M_Words.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\word-tester\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C678FE01-E60E-4E03-B0AB-6BECF9843977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1EFBF04-C69E-45C6-9F15-DDBF2E97AF9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A78F504C-B3D1-44D7-A0F0-C4A481C15F08}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="207">
   <si>
     <t>단어 (Word)</t>
   </si>
@@ -465,18 +465,12 @@
     <t>2) In the keeping of the police; in jail</t>
   </si>
   <si>
-    <t>degrade [v.]</t>
-  </si>
-  <si>
     <t>To bring shame or disgrace upon</t>
   </si>
   <si>
     <t>Causing shame or disgrace</t>
   </si>
   <si>
-    <t>detain [v.]</t>
-  </si>
-  <si>
     <t>To stop or hold; to keep from going on</t>
   </si>
   <si>
@@ -504,9 +498,6 @@
     <t>• The property extends for a half mile beyond the river.</t>
   </si>
   <si>
-    <t>integrate [v.]</t>
-  </si>
-  <si>
     <t>To unite into a whole; especially to end the separation of people of different races</t>
   </si>
   <si>
@@ -534,9 +525,6 @@
     <t>• The team felt triumphant after winning the championship game.</t>
   </si>
   <si>
-    <t>vacate [v.]</t>
-  </si>
-  <si>
     <t>To make empty, as by leaving</t>
   </si>
   <si>
@@ -624,82 +612,74 @@
     <t>• The hall monitor detained us until we could prove we had permission to leave the classroom. • The police had to detain the suspect to ask him more questions. • The meeting was supposed to end at 3 p.m., but several questions detained us.</t>
   </si>
   <si>
-    <t>extend [v.] (Sense 1)</t>
-  </si>
-  <si>
-    <t>extend [v.] (Sense 2)</t>
-  </si>
-  <si>
-    <t>extend [v.] (Sense 3)</t>
-  </si>
-  <si>
-    <t>extend [v.] (Sense 4)</t>
-  </si>
-  <si>
     <t>• The town worked hard to integrate people from different cultures and backgrounds. • We need to integrate all of our ideas to create one final project.</t>
   </si>
   <si>
-    <t>triumph [n.] (Sense 1)</t>
-  </si>
-  <si>
-    <t>triumph [n.] (Sense 2)</t>
-  </si>
-  <si>
     <t>• We will vacate the house at the end of June to make way for the people moving in. • The hotel asked guests to vacate their rooms by 11 a.m. on the day of departure. • During the evacuation drill, everyone practiced how to vacate the building quickly and safely. • The teacher asked the students to vacate their desks during the classroom renovation.</t>
   </si>
   <si>
-    <t>verdict [n.] (Sense 1)</t>
-  </si>
-  <si>
     <t>• The jury looked grim as she announced the verdict. • The jury gave a verdict of "guilty" after hearing all the evidence in the trial.</t>
   </si>
   <si>
-    <t>verdict [n.] (Sense 2)</t>
-  </si>
-  <si>
     <t>• The verdict on the new computer is that it does twice the work in half the time. • After the game, the coach gave his verdict on how the team performed.</t>
   </si>
   <si>
-    <t>violate [v.] (Sense 1)</t>
-  </si>
-  <si>
     <t>• Damien violated our teacher’s trust by trying to cheat on the homework. • If you talk during a test, you might violate the rules of the classroom.</t>
   </si>
   <si>
-    <t>violate [v.] (Sense 2)</t>
-  </si>
-  <si>
-    <t>break up (Sense 1)</t>
-  </si>
-  <si>
-    <t>break up (Sense 2)</t>
-  </si>
-  <si>
-    <t>break up (Sense 3)</t>
-  </si>
-  <si>
-    <t>bring back (Sense 1)</t>
-  </si>
-  <si>
-    <t>bring back (Sense 2)</t>
-  </si>
-  <si>
-    <t>bring back (Sense 3)</t>
-  </si>
-  <si>
     <t xml:space="preserve">arrogance [n.]  </t>
   </si>
   <si>
-    <t xml:space="preserve">degrading [adj.]  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">triumph [v.]  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">triumphant [adj.]  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">violation [n.]  </t>
+    <t>degrade</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>degrading</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>detain</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>extend</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>integrate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>triumph</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>triumphant</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>vacate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>verdict</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>violate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>violation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>break up</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>bring back</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1630,12 +1610,12 @@
         <v>126</v>
       </c>
       <c r="C2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>213</v>
+        <v>193</v>
       </c>
       <c r="B3" t="s">
         <v>127</v>
@@ -1674,183 +1654,183 @@
         <v>136</v>
       </c>
       <c r="C6" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B7" t="s">
         <v>137</v>
       </c>
       <c r="C7" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B8" t="s">
         <v>138</v>
       </c>
       <c r="C8" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>194</v>
+      </c>
+      <c r="B9" t="s">
         <v>139</v>
       </c>
-      <c r="B9" t="s">
-        <v>140</v>
-      </c>
       <c r="C9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>214</v>
+        <v>195</v>
       </c>
       <c r="B10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C10" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>142</v>
+        <v>196</v>
       </c>
       <c r="B11" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C11" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="B12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C12" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="B13" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C13" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B14" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C14" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B15" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>152</v>
+        <v>198</v>
       </c>
       <c r="B16" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C16" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B17" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C17" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B18" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C18" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="B19" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C19" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="B20" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C20" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>162</v>
+        <v>201</v>
       </c>
       <c r="B21" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C21" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B22" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C22" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -1858,109 +1838,109 @@
         <v>202</v>
       </c>
       <c r="B23" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C23" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B24" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C24" t="s">
-        <v>205</v>
+        <v>192</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B25" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C25" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>217</v>
+        <v>204</v>
       </c>
       <c r="B26" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C26" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B27" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C27" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B28" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C28" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="B29" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C29" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B30" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C30" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="B31" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C31" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="B32" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C32" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove part of speech from an excel file 2
</commit_message>
<xml_diff>
--- a/data/2026_F_M_Words.xlsx
+++ b/data/2026_F_M_Words.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\word-tester\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1EFBF04-C69E-45C6-9F15-DDBF2E97AF9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{164F8DEA-1FB9-4833-95CB-DEB960CAFF5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A78F504C-B3D1-44D7-A0F0-C4A481C15F08}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="206">
   <si>
     <t>단어 (Word)</t>
   </si>
@@ -423,9 +423,6 @@
     <t>뜻 (Definition)</t>
   </si>
   <si>
-    <t>arrogant [adj.]</t>
-  </si>
-  <si>
     <t>Showing too much pride in oneself</t>
   </si>
   <si>
@@ -435,27 +432,18 @@
     <t>• Declaring that you are sure to win is another example of your arrogance.</t>
   </si>
   <si>
-    <t>boycott [v.]</t>
-  </si>
-  <si>
     <t>To join others in refusing to support an organization</t>
   </si>
   <si>
     <t>• Customers plan to boycott that store if it continues to discriminate.</t>
   </si>
   <si>
-    <t>campaign [v.]</t>
-  </si>
-  <si>
     <t>To take part in actions planned to accomplish a particular goal</t>
   </si>
   <si>
     <t>• Students who wish to campaign for class office must submit petitions.</t>
   </si>
   <si>
-    <t>ceremony [n.]</t>
-  </si>
-  <si>
     <t>A formal event held in honor of a special occasion.</t>
   </si>
   <si>
@@ -591,15 +579,9 @@
     <t>• The bride and groom exchanged rings during the wedding ceremony. • The graduation ceremony will take place in the school gym next week. • There will be a ceremony to honor the firefighters for their bravery.</t>
   </si>
   <si>
-    <t>custody [n.] (Sense 1)</t>
-  </si>
-  <si>
     <t>• The stolen Picasso painting was returned to the custody of the Museum of Modern Art. • After their parents separated, the court decided who would have custody of the children.</t>
   </si>
   <si>
-    <t>custody [n.] (Sense 2)</t>
-  </si>
-  <si>
     <t>• The police officer took the thief into custody. • After the accident, the authorities took custody of the evidence for investigation.</t>
   </si>
   <si>
@@ -627,9 +609,6 @@
     <t>• Damien violated our teacher’s trust by trying to cheat on the homework. • If you talk during a test, you might violate the rules of the classroom.</t>
   </si>
   <si>
-    <t xml:space="preserve">arrogance [n.]  </t>
-  </si>
-  <si>
     <t>degrade</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -679,6 +658,30 @@
   </si>
   <si>
     <t>bring back</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>arrogant</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>arrogance</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>boycott</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>campaign</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ceremony</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>custody</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1604,343 +1607,343 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B2" t="s">
         <v>125</v>
       </c>
-      <c r="B2" t="s">
-        <v>126</v>
-      </c>
       <c r="C2" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="B3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C3" t="s">
         <v>127</v>
-      </c>
-      <c r="C3" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>202</v>
+      </c>
+      <c r="B4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C4" t="s">
         <v>129</v>
-      </c>
-      <c r="B4" t="s">
-        <v>130</v>
-      </c>
-      <c r="C4" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>132</v>
+        <v>203</v>
       </c>
       <c r="B5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C5" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>135</v>
+        <v>204</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C6" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>181</v>
+        <v>205</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C7" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>183</v>
+        <v>205</v>
       </c>
       <c r="B8" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C8" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="B9" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C9" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="B10" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C10" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="B11" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C11" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B12" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C12" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B13" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C13" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B14" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C14" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B15" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C15" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="B16" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C16" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="B17" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C17" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="B18" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C18" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="B19" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C19" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="B20" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C20" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="B21" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C21" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B22" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C22" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B23" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C23" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="B24" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C24" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="B25" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C25" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="B26" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C26" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="B27" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C27" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="B28" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C28" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="B29" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C29" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="B30" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C30" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="B31" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C31" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="B32" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C32" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>